<commit_message>
TABLA usuario_productos DEF EXCEL
</commit_message>
<xml_diff>
--- a/BasesDatos/Tabla1_tienda_productos.xlsx
+++ b/BasesDatos/Tabla1_tienda_productos.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Documents\1_ISIC\7_Semestre\GPS\WiseAgend\BasesDatos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Documents\WiseAgend\BasesDatos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{113636DC-E365-4DAD-B792-5C9723EF24BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB726B70-AECE-4076-8D47-1FBAB7248301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-115" yWindow="-115" windowWidth="24697" windowHeight="14795" xr2:uid="{F4BDB6D1-DAD1-4C0D-B66F-9056E19386D0}"/>
+    <workbookView xWindow="3326" yWindow="3326" windowWidth="18350" windowHeight="10615" xr2:uid="{F4BDB6D1-DAD1-4C0D-B66F-9056E19386D0}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="51">
   <si>
     <t>Campo</t>
   </si>
@@ -323,16 +323,49 @@
     <t>TABLA tienda_productos</t>
   </si>
   <si>
-    <t>id_recompensas</t>
-  </si>
-  <si>
-    <t>nombre_recompensas</t>
-  </si>
-  <si>
-    <t>valor_tokens</t>
-  </si>
-  <si>
-    <t>preiodo_vencimiento</t>
+    <t>Fecha y hora de la transacción (compra o canje).</t>
+  </si>
+  <si>
+    <t>DEFAULT CURRENT_TIMESTAMP</t>
+  </si>
+  <si>
+    <t>DATETIME</t>
+  </si>
+  <si>
+    <t>fecha_compra</t>
+  </si>
+  <si>
+    <t>FK &gt; tienda_productos(id_producto). Identificador del producto comprado/canjeado.</t>
+  </si>
+  <si>
+    <t>id_producto</t>
+  </si>
+  <si>
+    <t>FK &gt; usuarios(id_usuario). Identificador del usuario que adquiere el producto.</t>
+  </si>
+  <si>
+    <t>id_usuario</t>
+  </si>
+  <si>
+    <t>Descripción</t>
+  </si>
+  <si>
+    <t>Restricción / Default</t>
+  </si>
+  <si>
+    <t>Tipo</t>
+  </si>
+  <si>
+    <t>usuarios_productos</t>
+  </si>
+  <si>
+    <t>nombre</t>
+  </si>
+  <si>
+    <t>costo</t>
+  </si>
+  <si>
+    <t>fecha_vencimiento</t>
   </si>
 </sst>
 </file>
@@ -527,77 +560,77 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -913,24 +946,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C06DBECA-98A6-4BE0-83E6-3B05C5F22E31}">
-  <dimension ref="A4:D19"/>
+  <dimension ref="A4:I19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.65" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="15.77734375" customWidth="1"/>
     <col min="3" max="3" width="19.88671875" customWidth="1"/>
     <col min="4" max="4" width="34.77734375" customWidth="1"/>
+    <col min="9" max="9" width="27.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="26" t="s">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="26"/>
-      <c r="C4" s="26"/>
-      <c r="D4" s="26"/>
-    </row>
-    <row r="5" spans="1:4" ht="15.3" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="F4" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="14"/>
+    </row>
+    <row r="5" spans="1:9" ht="23.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -943,169 +983,218 @@
       <c r="D5" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="24.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B6" s="4" t="s">
+      <c r="F5" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="81.599999999999994" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="23.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B7" s="7" t="s">
+      <c r="F6" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="80.95" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="6" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="38.25" x14ac:dyDescent="0.3">
+      <c r="F7" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="58" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="7" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="14"/>
-      <c r="B9" s="18"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="10" t="s">
+      <c r="F8" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" s="16"/>
+      <c r="B9" s="19"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="14"/>
-      <c r="B10" s="18"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="9" t="s">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10" s="16"/>
+      <c r="B10" s="19"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="15.3" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="16"/>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="5" t="s">
+    <row r="11" spans="1:9" ht="15.3" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="17"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="23.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B12" s="7" t="s">
+    <row r="12" spans="1:9" ht="23.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="B12" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="15.3" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="3" t="s">
+    <row r="13" spans="1:9" ht="15.3" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="35.049999999999997" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B14" s="7" t="s">
+    <row r="14" spans="1:9" ht="35.049999999999997" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="12" t="s">
+      <c r="C14" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="6" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="35.049999999999997" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="3" t="s">
+    <row r="15" spans="1:9" ht="35.049999999999997" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="B16" s="23" t="s">
+      <c r="B16" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="C16" s="23" t="s">
+      <c r="C16" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="D16" s="13" t="s">
+      <c r="D16" s="11" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="20"/>
-      <c r="B17" s="24"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="13" t="s">
+      <c r="A17" s="22"/>
+      <c r="B17" s="25"/>
+      <c r="C17" s="25"/>
+      <c r="D17" s="11" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="22.95" x14ac:dyDescent="0.3">
-      <c r="A18" s="20"/>
-      <c r="B18" s="24"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="13" t="s">
+      <c r="A18" s="22"/>
+      <c r="B18" s="25"/>
+      <c r="C18" s="25"/>
+      <c r="D18" s="11" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="23.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="22"/>
-      <c r="B19" s="25"/>
-      <c r="C19" s="25"/>
-      <c r="D19" s="8" t="s">
+      <c r="A19" s="23"/>
+      <c r="B19" s="26"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="6" t="s">
         <v>34</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
+    <mergeCell ref="F4:I4"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A8:A11"/>
     <mergeCell ref="B8:B11"/>

</xml_diff>